<commit_message>
Updated Data Samples and retested the program
</commit_message>
<xml_diff>
--- a/outputs/model_comparison.xlsx
+++ b/outputs/model_comparison.xlsx
@@ -462,16 +462,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.775</v>
       </c>
       <c r="C2" t="n">
-        <v>81.81818181818183</v>
+        <v>77.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7878787878787878</v>
+        <v>0.7333333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3</v>
       </c>
       <c r="C3" t="n">
-        <v>18.18181818181818</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1066666666666667</v>
+        <v>0.2123809523809524</v>
       </c>
       <c r="E3" t="n">
-        <v>0.09696969696969697</v>
+        <v>0.2225</v>
       </c>
     </row>
     <row r="4">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.225</v>
       </c>
       <c r="C4" t="n">
-        <v>36.36363636363637</v>
+        <v>22.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.35</v>
+        <v>0.1809523809523809</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -519,16 +519,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.8</v>
       </c>
       <c r="C5" t="n">
-        <v>81.81818181818183</v>
+        <v>80</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8</v>
+        <v>0.7371428571428572</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7878787878787878</v>
+        <v>0.7566666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>